<commit_message>
Current state. Doesn't match main TIMES model
</commit_message>
<xml_diff>
--- a/kea-times-model/SubRES_TMPL/SubRES_NewTech_AGR_KEA_Trans.xlsx
+++ b/kea-times-model/SubRES_TMPL/SubRES_NewTech_AGR_KEA_Trans.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cattonw\git\TIMES-NZ-Model-Files\kea-times-model\SubRES_TMPL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\weerasa\TIMES-NZ-Model-Files\TIMES-NZ\SubRES_TMPL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{03D9A797-6862-4931-817F-712EE73C22AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07078184-DF4B-4BAC-933D-3EEFEC76ADD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="21600" windowHeight="11295" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Documentation" sheetId="20" r:id="rId1"/>
@@ -696,24 +696,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24CB2892-F0CC-4065-A68A-8171F2DE7F2C}">
   <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>37</v>
       </c>
@@ -726,21 +726,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B3:E16"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.7109375" customWidth="1"/>
-    <col min="2" max="2" width="31.85546875" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.7265625" customWidth="1"/>
+    <col min="2" max="2" width="31.81640625" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:5" ht="13" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="5" t="s">
         <v>6</v>
       </c>
@@ -754,7 +754,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>23</v>
       </c>
@@ -762,7 +762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
         <v>33</v>
       </c>
@@ -770,7 +770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="D16" s="11"/>
     </row>
   </sheetData>
@@ -783,34 +783,34 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B3:P15"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="2.85546875" customWidth="1"/>
-    <col min="2" max="2" width="11.5703125" customWidth="1"/>
-    <col min="3" max="4" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="2.81640625" customWidth="1"/>
+    <col min="2" max="2" width="11.54296875" customWidth="1"/>
+    <col min="3" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="10.7265625" customWidth="1"/>
     <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.1796875" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="9" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.85546875" customWidth="1"/>
-    <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.81640625" customWidth="1"/>
+    <col min="18" max="18" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.54296875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:16" ht="15" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:16" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>0</v>
       </c>
@@ -823,7 +823,7 @@
       <c r="O5" s="1"/>
       <c r="P5" s="1"/>
     </row>
-    <row r="6" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="I6" s="2"/>
       <c r="J6" s="1"/>
@@ -834,7 +834,7 @@
       <c r="O6" s="1"/>
       <c r="P6" s="1"/>
     </row>
-    <row r="7" spans="2:16" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:16" ht="13.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="4" t="s">
         <v>1</v>
       </c>
@@ -881,7 +881,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B8" s="11" t="s">
         <v>24</v>
       </c>
@@ -901,7 +901,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B9" s="11" t="s">
         <v>27</v>
       </c>
@@ -921,7 +921,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B10" s="11" t="s">
         <v>28</v>
       </c>
@@ -941,7 +941,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B11" s="11" t="s">
         <v>29</v>
       </c>
@@ -961,7 +961,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
         <v>24</v>
       </c>
@@ -981,7 +981,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B13" s="11" t="s">
         <v>27</v>
       </c>
@@ -1001,7 +1001,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B14" s="11" t="s">
         <v>28</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B15" s="11" t="s">
         <v>29</v>
       </c>
@@ -1053,29 +1053,29 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B2:N4"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.5703125" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.54296875" customWidth="1"/>
+    <col min="2" max="2" width="26.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.1796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="10.7265625" customWidth="1"/>
+    <col min="13" max="13" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:14" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:14" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:14" ht="13" x14ac:dyDescent="0.3">
       <c r="B4" s="8" t="s">
         <v>16</v>
       </c>

</xml_diff>